<commit_message>
docs(acquisition): resolve placeholder SharePoint folders by NbS in the hand-off files
</commit_message>
<xml_diff>
--- a/methodology/decisions/2026-10-07_acquisition_handoff.xlsx
+++ b/methodology/decisions/2026-10-07_acquisition_handoff.xlsx
@@ -582,11 +582,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr"/>
@@ -770,7 +766,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/abasse_2023_fmnr_niger_state_of_knowledge.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/abasse_2023_fmnr_niger_state_of_knowledge.pdf</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -778,8 +774,6 @@
           <t>abasse_2023_fmnr_niger_state_of_knowledge.pdf</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -829,7 +823,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/abdulai_2018_cocoa_af_less_resilient.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/abdulai_2018_cocoa_af_less_resilient.pdf</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -837,8 +831,6 @@
           <t>abdulai_2018_cocoa_af_less_resilient.pdf</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -888,7 +880,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/baker_2025.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/baker_2025.pdf</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -896,8 +888,6 @@
           <t>baker_2025.pdf</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -947,7 +937,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bayala_2014_parklands_buffering_climate_risk.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/bayala_2014_parklands_buffering_climate_risk.pdf</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -955,8 +945,6 @@
           <t>bayala_2014_parklands_buffering_climate_risk.pdf</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -994,7 +982,6 @@
           <t>Bayard et al. (2007). The economics of adoption and management of alley cropping in Haiti. Journal of Environmental Management.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jenvman.2006.05.001</t>
@@ -1010,8 +997,6 @@
           <t>bayard2006_haiti_alleycrop_econ.pdf</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>paywalled_elsevier</t>
@@ -1069,8 +1054,6 @@
           <t>beefcattle2024_heatstress.pdf</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>paywalled (Springer)</t>
@@ -1120,7 +1103,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/begum_2025.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/begum_2025.pdf</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1128,8 +1111,6 @@
           <t>begum_2025.pdf</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1179,7 +1160,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/botoni_2010_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/botoni_2010_fr.pdf</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1187,8 +1168,6 @@
           <t>botoni_2010_fr.pdf</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1246,8 +1225,6 @@
           <t>caatinga2022_thermalcomfort_arrangements.pdf</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>paywalled (Springer)</t>
@@ -1297,7 +1274,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/cardinael_2018.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/cardinael_2018.pdf</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1305,8 +1282,6 @@
           <t>cardinael_2018.pdf</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1356,7 +1331,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/chaudhury_2011_icraf_wp_zambia_honduras.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/chaudhury_2011_icraf_wp_zambia_honduras.pdf</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1364,8 +1339,6 @@
           <t>chaudhury_2011_icraf_wp_zambia_honduras.pdf</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -1415,7 +1388,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/guaqueta_2025_silvopastoral_el_nino_colombia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/guaqueta_2025_silvopastoral_el_nino_colombia.pdf</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1423,8 +1396,6 @@
           <t>guaqueta_2025_silvopastoral_el_nino_colombia.pdf</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -1474,7 +1445,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/hao_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/hao_2026.pdf</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1482,8 +1453,6 @@
           <t>hao_2026.pdf</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1533,7 +1502,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/haverhals_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/haverhals_2016.pdf</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1541,8 +1510,6 @@
           <t>haverhals_2016.pdf</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1600,8 +1567,6 @@
           <t>homegarden_carbon_storage_2022.pdf</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>paywalled (Elsevier)</t>
@@ -1651,7 +1616,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/niether_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/niether_2020.pdf</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1659,8 +1624,6 @@
           <t>niether_2020.pdf</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1710,7 +1673,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ntawuruhunga_2023.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/ntawuruhunga_2023.pdf</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1718,8 +1681,6 @@
           <t>ntawuruhunga_2023.pdf</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1769,7 +1730,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/pumarino_2015.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/pumarino_2015.pdf</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1777,8 +1738,6 @@
           <t>pumarino_2015.pdf</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1816,7 +1775,6 @@
           <t>Robusti, E.A.; Zapparoli, I.D.; Santoro, P.H. (2017). Café arborizado no Estado do Paraná, Brasil: indicadores financeiros e interferências ambientais, 2012-2014. Agroalimentaria, 23(44), 79-91.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
           <t>https://www.redalyc.org/journal/1992/199252873006/html/</t>
@@ -1824,7 +1782,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/robusti_2017_pt.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/robusti_2017_pt.pdf</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1832,8 +1790,6 @@
           <t>robusti_2017_pt.pdf</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1883,7 +1839,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sanchez_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/sanchez_2026.pdf</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1891,8 +1847,6 @@
           <t>sanchez_2026.pdf</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -1942,7 +1896,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sharma_2022.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/sharma_2022.pdf</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1950,8 +1904,6 @@
           <t>sharma_2022.pdf</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -2001,7 +1953,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/solorio_2016_silvopastoral_drought_chapter.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/solorio_2016_silvopastoral_drought_chapter.pdf</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2009,8 +1961,6 @@
           <t>solorio_2016_silvopastoral_drought_chapter.pdf</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2048,7 +1998,6 @@
           <t>Vaast P. &amp; Somarriba E. (2014/2016). Shaded coffee and cocoa – double dividend for biodiversity and small-scale farmers. Ecological Economics / Agroforestry Systems.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
           <t>https://www.cifor.org/knowledge/publication/5553</t>
@@ -2064,8 +2013,6 @@
           <t>vaast2016_double_dividend.pdf</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>OA (Unpaywall:repository)</t>
@@ -2115,7 +2062,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/zhu_2019.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/zhu_2019.pdf</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2123,8 +2070,6 @@
           <t>zhu_2019.pdf</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>landing page only (no citation_pdf_url / Unpaywall pdf) — human browser download</t>
@@ -2174,7 +2119,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/badji_2013_mise_en_defens_senegal.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/badji_2013_mise_en_defens_senegal.pdf</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2182,8 +2127,6 @@
           <t>badji_2013_mise_en_defens_senegal.pdf</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2233,7 +2176,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/barajas_guzman_2013_acolchados_reforestacion_costos.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/barajas_guzman_2013_acolchados_reforestacion_costos.pdf</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2241,8 +2184,6 @@
           <t>barajas_guzman_2013_acolchados_reforestacion_costos.pdf</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2292,7 +2233,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bradshaw_2007_deforestation_flood_risk.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/bradshaw_2007_deforestation_flood_risk.pdf</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2300,8 +2241,6 @@
           <t>bradshaw_2007_deforestation_flood_risk.pdf</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2351,7 +2290,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/brancalion_2019_restoration_costs_brazil.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/brancalion_2019_restoration_costs_brazil.pdf</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2359,8 +2298,6 @@
           <t>brancalion_2019_restoration_costs_brazil.pdf</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2410,7 +2347,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/das_vincent_2009_mangroves_super_cyclone.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/das_vincent_2009_mangroves_super_cyclone.pdf</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2418,8 +2355,6 @@
           <t>das_vincent_2009_mangroves_super_cyclone.pdf</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2469,7 +2404,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/del_valle_2020_mangroves_economic_activity_hurricanes.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/del_valle_2020_mangroves_economic_activity_hurricanes.pdf</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2477,8 +2412,6 @@
           <t>del_valle_2020_mangroves_economic_activity_hurricanes.pdf</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2528,7 +2461,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/didy_2026_mangroves_sainte_marie_reboisement_vs_rna.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/didy_2026_mangroves_sainte_marie_reboisement_vs_rna.pdf</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2536,8 +2469,6 @@
           <t>didy_2026_mangroves_sainte_marie_reboisement_vs_rna.pdf</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -2595,8 +2526,6 @@
           <t>enrichment_planting_seedling_survival_tradeoffs_2018.pdf</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>paywalled (closed, UW Press)</t>
@@ -2634,7 +2563,6 @@
           <t>FAO; CIFOR (2005). Forests and floods: drowning in fiction or thriving on facts? RAP Publication 2005/03, Forest Perspectives 2. FAO Regional Office for Asia and the Pacific / CIFOR, Bangkok/Bogor.</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
           <t>https://www.cifor.org/library/1738/forests-and-floods-drowning-in-fiction-or-thriving-on-facts/</t>
@@ -2642,7 +2570,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/fao_cifor_2005_forests_floods.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/fao_cifor_2005_forests_floods.pdf</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2650,8 +2578,6 @@
           <t>fao_cifor_2005_forests_floods.pdf</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2701,7 +2627,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/farley_2005_afforestation_water_yield.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/farley_2005_afforestation_water_yield.pdf</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2709,8 +2635,6 @@
           <t>farley_2005_afforestation_water_yield.pdf</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -2768,8 +2692,6 @@
           <t>fr_nucleation_seedling_planting_2024.pdf</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>paywalled (Wiley, oa_status=closed)</t>
@@ -2819,7 +2741,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/gardiner_2021_wind_damage_planted_forests.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/gardiner_2021_wind_damage_planted_forests.pdf</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2827,8 +2749,6 @@
           <t>gardiner_2021_wind_damage_planted_forests.pdf</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2878,7 +2798,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/gorman_2022_planted_mangrove_survival.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/gorman_2022_planted_mangrove_survival.pdf</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,8 +2806,6 @@
           <t>gorman_2022_planted_mangrove_survival.pdf</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2937,7 +2855,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/hajjar_2021_community_forests_global.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/hajjar_2021_community_forests_global.pdf</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2945,8 +2863,6 @@
           <t>hajjar_2021_community_forests_global.pdf</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -2996,7 +2912,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/herath_2025_forest_cover_flood_sr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/herath_2025_forest_cover_flood_sr.pdf</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3004,8 +2920,6 @@
           <t>herath_2025_forest_cover_flood_sr.pdf</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3055,7 +2969,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/hochard_2019_mangroves_economic_activity_cyclones.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/hochard_2019_mangroves_economic_activity_cyclones.pdf</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3063,8 +2977,6 @@
           <t>hochard_2019_mangroves_economic_activity_cyclones.pdf</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3102,7 +3014,6 @@
           <t>Independent Evaluation Group (2013). Managing Forest Resources for Sustainable Development: An Evaluation of World Bank Group Experience. World Bank, Washington DC.</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
           <t>https://ieg.worldbankgroup.org/evaluations/managing-forest-resources-sustainable-development</t>
@@ -3110,7 +3021,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ieg_2013_managing_forest_resources.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/ieg_2013_managing_forest_resources.pdf</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3118,8 +3029,6 @@
           <t>ieg_2013_managing_forest_resources.pdf</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3157,7 +3066,6 @@
           <t>Independent Evaluation Group (2018). Vietnam - Forest Sector Development Project. Project Performance Assessment Report No. 123895. World Bank, Washington DC.</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
           <t>https://ieg.worldbankgroup.org/reports/vietnam-forest-sector-development-project</t>
@@ -3165,7 +3073,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ieg_2018_ppar_vietnam_forest_sector.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/ieg_2018_ppar_vietnam_forest_sector.pdf</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3173,8 +3081,6 @@
           <t>ieg_2018_ppar_vietnam_forest_sector.pdf</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3212,7 +3118,6 @@
           <t>Vira, B., Wildburger, C., Mansourian, S. (eds.) (2015). Forests, Trees and Landscapes for Food Security and Nutrition: A Global Assessment Report. IUFRO World Series Vol. 33. IUFRO, Vienna.</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
           <t>https://cgspace.cgiar.org/handle/10568/94088</t>
@@ -3220,7 +3125,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/iufro_2015_gfep_food_security.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/iufro_2015_gfep_food_security.pdf</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3228,8 +3133,6 @@
           <t>iufro_2015_gfep_food_security.pdf</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3279,7 +3182,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kandel_2022_pa_household_income_meta.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/kandel_2022_pa_household_income_meta.pdf</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3287,8 +3190,6 @@
           <t>kandel_2022_pa_household_income_meta.pdf</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -3338,7 +3239,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kimwanga_2026_forest_comanagement_rainfall_shocks.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/kimwanga_2026_forest_comanagement_rainfall_shocks.pdf</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3346,8 +3247,6 @@
           <t>kimwanga_2026_forest_comanagement_rainfall_shocks.pdf</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3397,7 +3296,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/mahmud_barbier_2016_defensive_expenditure_bangladesh.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/mahmud_barbier_2016_defensive_expenditure_bangladesh.pdf</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3405,8 +3304,6 @@
           <t>mahmud_barbier_2016_defensive_expenditure_bangladesh.pdf</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3456,7 +3353,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/marois_mitsch_2015_mangrove_tsunami_cyclone.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/marois_mitsch_2015_mangrove_tsunami_cyclone.pdf</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3464,8 +3361,6 @@
           <t>marois_mitsch_2015_mangrove_tsunami_cyclone.pdf</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3515,7 +3410,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/naidoo_2019_protected_areas_wellbeing.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/naidoo_2019_protected_areas_wellbeing.pdf</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3523,8 +3418,6 @@
           <t>naidoo_2019_protected_areas_wellbeing.pdf</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3574,7 +3467,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/nunes_silva_2020_custos_restauracao_itacaiunas.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/nunes_silva_2020_custos_restauracao_itacaiunas.pdf</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3582,8 +3475,6 @@
           <t>nunes_silva_2020_custos_restauracao_itacaiunas.pdf</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -3641,8 +3532,6 @@
           <t>reforestation_drought_west_africa_2017.pdf</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>paywalled (closed, Springer)</t>
@@ -3692,7 +3581,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/robertson_wunder_2005_huellas_frescas_psa_bolivia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/robertson_wunder_2005_huellas_frescas_psa_bolivia.pdf</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3700,8 +3589,6 @@
           <t>robertson_wunder_2005_huellas_frescas_psa_bolivia.pdf</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3751,7 +3638,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/rojas_2011_psa_plantaciones_costa_rica.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/rojas_2011_psa_plantaciones_costa_rica.pdf</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3759,8 +3646,6 @@
           <t>rojas_2011_psa_plantaciones_costa_rica.pdf</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3810,7 +3695,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/samii_2014_dfm_campbell.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/samii_2014_dfm_campbell.pdf</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3818,8 +3703,6 @@
           <t>samii_2014_dfm_campbell.pdf</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3877,8 +3760,6 @@
           <t>sierra_planting_vs_natural_1978.pdf</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t xml:space="preserve">WRONG PDF acquired (cached + SharePoint copy = Donato, Campbell &amp; Franklin 2012, J Veg Sci, doi 10.1111/j.1654-1103.2011.01362.x) — re-acquire Bock et al. 1978 </t>
@@ -3928,7 +3809,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/snilstveit_2019_pes_climate_campbell.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/snilstveit_2019_pes_climate_campbell.pdf</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3936,8 +3817,6 @@
           <t>snilstveit_2019_pes_climate_campbell.pdf</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -3987,7 +3866,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/vandijk_2009_forest_flood_tenuous.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/vandijk_2009_forest_flood_tenuous.pdf</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3995,8 +3874,6 @@
           <t>vandijk_2009_forest_flood_tenuous.pdf</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -4046,7 +3923,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/yang_2023_vegrestoration_erosion_meta.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/yang_2023_vegrestoration_erosion_meta.pdf</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4054,8 +3931,6 @@
           <t>yang_2023_vegrestoration_erosion_meta.pdf</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -4113,8 +3988,6 @@
           <t>critical_source_areas_buffer_planning_2009.pdf</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>Springer paywall</t>
@@ -4164,7 +4037,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/arslan_2015_csa_zambia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/arslan_2015_csa_zambia.pdf</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4172,8 +4045,6 @@
           <t>arslan_2015_csa_zambia.pdf</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4223,7 +4094,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/biazin_2012.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/biazin_2012.pdf</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4231,8 +4102,6 @@
           <t>biazin_2012.pdf</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4282,7 +4151,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/boillat_2019_ca_buffer_rainfall_variability.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/boillat_2019_ca_buffer_rainfall_variability.pdf</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4290,8 +4159,6 @@
           <t>boillat_2019_ca_buffer_rainfall_variability.pdf</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4341,7 +4208,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bruelle_2014_ca_upland_rice_variability.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/bruelle_2014_ca_upland_rice_variability.pdf</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4349,8 +4216,6 @@
           <t>bruelle_2014_ca_upland_rice_variability.pdf</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4408,8 +4273,6 @@
           <t>checkdam_runoff_sediment_semiarid_2014.pdf</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>paywalled (JSWC / SWCS)</t>
@@ -4467,8 +4330,6 @@
           <t>checkdams_runoff_sediment_loess_2019.pdf</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
           <t>paywalled (Elsevier)</t>
@@ -4518,7 +4379,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/corbeels_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/corbeels_2020.pdf</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4526,8 +4387,6 @@
           <t>corbeels_2020.pdf</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4577,7 +4436,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_an0083_sime_2015.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_an0083_sime_2015.pdf</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4585,8 +4444,6 @@
           <t>era_an0083_sime_2015.pdf</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4636,7 +4493,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_an0121_wang_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_an0121_wang_2016.pdf</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4644,8 +4501,6 @@
           <t>era_an0121_wang_2016.pdf</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4695,7 +4550,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_dk0008_dalton_2014.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_dk0008_dalton_2014.pdf</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4703,8 +4558,6 @@
           <t>era_dk0008_dalton_2014.pdf</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4754,7 +4607,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_hk0259_umar_2012.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_hk0259_umar_2012.pdf</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4762,8 +4615,6 @@
           <t>era_hk0259_umar_2012.pdf</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4813,7 +4664,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_js0241_adgo_2013.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_js0241_adgo_2013.pdf</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4821,8 +4672,6 @@
           <t>era_js0241_adgo_2013.pdf</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4872,7 +4721,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_nn0102_chiroma_2006.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_nn0102_chiroma_2006.pdf</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4880,8 +4729,6 @@
           <t>era_nn0102_chiroma_2006.pdf</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4931,7 +4778,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_nn0259_fox_2005.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_nn0259_fox_2005.pdf</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4939,8 +4786,6 @@
           <t>era_nn0259_fox_2005.pdf</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -4990,7 +4835,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_nn0305_mazvimavi_2009.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_nn0305_mazvimavi_2009.pdf</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4998,8 +4843,6 @@
           <t>era_nn0305_mazvimavi_2009.pdf</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5049,7 +4892,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_nn0385_mo_2017.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_nn0385_mo_2017.pdf</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5057,8 +4900,6 @@
           <t>era_nn0385_mo_2017.pdf</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5108,7 +4949,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/fan_2023.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/fan_2023.pdf</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5116,8 +4957,6 @@
           <t>fan_2023.pdf</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5167,7 +5006,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/gebremeskel_2018.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/gebremeskel_2018.pdf</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5175,8 +5014,6 @@
           <t>gebremeskel_2018.pdf</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
           <t>paywalled (verified: Unpaywall + web search found no copy) → institutional</t>
@@ -5226,7 +5063,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/gonzalezsanchez_2019.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/gonzalezsanchez_2019.pdf</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5234,8 +5071,6 @@
           <t>gonzalezsanchez_2019.pdf</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5285,7 +5120,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/lucasborja_2021.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/lucasborja_2021.pdf</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5293,8 +5128,6 @@
           <t>lucasborja_2021.pdf</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5344,7 +5177,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/makmensah_2021.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/makmensah_2021.pdf</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5352,8 +5185,6 @@
           <t>makmensah_2021.pdf</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5403,7 +5234,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/mashavakure_2025_ca_el_nino_zimbabwe.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/mashavakure_2025_ca_el_nino_zimbabwe.pdf</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5411,8 +5242,6 @@
           <t>mashavakure_2025_ca_el_nino_zimbabwe.pdf</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5462,7 +5291,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/mekonnen_2014.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/mekonnen_2014.pdf</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5470,8 +5299,6 @@
           <t>mekonnen_2014.pdf</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5521,7 +5348,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/michler_2019_ca_climate_resilience.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/michler_2019_ca_climate_resilience.pdf</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5529,8 +5356,6 @@
           <t>michler_2019_ca_climate_resilience.pdf</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5568,7 +5393,6 @@
           <t>Miranda, R.A. de (resp.) (2019). Relatório de avaliação dos impactos de tecnologias geradas pela Embrapa: Mini-barragens de contenção de águas superficiais de chuvas - Barraginhas (ano de avaliação 2018). Sete Lagoas: Em</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" s="5" t="inlineStr">
         <is>
           <t>https://bs.sede.embrapa.br/2018/relatorios/milhoesorgo_2018_minibarragens.pdf</t>
@@ -5576,7 +5400,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/miranda_2019_embrapa_barraginhas_pt.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/miranda_2019_embrapa_barraginhas_pt.pdf</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5584,8 +5408,6 @@
           <t>miranda_2019_embrapa_barraginhas_pt.pdf</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5635,7 +5457,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/moges_2011.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/moges_2011.pdf</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5643,8 +5465,6 @@
           <t>moges_2011.pdf</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5694,7 +5514,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ndungu_2023_tied_ridging_erratic_rainfall.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/ndungu_2023_tied_ridging_erratic_rainfall.pdf</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5702,8 +5522,6 @@
           <t>ndungu_2023_tied_ridging_erratic_rainfall.pdf</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5753,7 +5571,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/nguru_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/nguru_2026.pdf</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5761,8 +5579,6 @@
           <t>nguru_2026.pdf</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5800,7 +5616,6 @@
           <t>Assessing crop yield benefits from in situ rainwater harvesting through contour ridges in semi-arid Zimbabwe. Physics and Chemistry of the Earth, 2013.</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" s="5" t="inlineStr">
         <is>
           <t>https://www.sciencedirect.com/science/article/abs/pii/S1474706513001253</t>
@@ -5816,8 +5631,6 @@
           <t>nyamadzawo_contour_ridges_zimbabwe_2013.pdf</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>wrong_pdf_in_library</t>
@@ -5867,7 +5680,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/palsaniya_2023_rwh_af_goat_india.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/palsaniya_2023_rwh_af_goat_india.pdf</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5875,8 +5688,6 @@
           <t>palsaniya_2023_rwh_af_goat_india.pdf</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5926,7 +5737,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/pittelkow_2015_when_notill_yields_more.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/pittelkow_2015_when_notill_yields_more.pdf</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -5934,8 +5745,6 @@
           <t>pittelkow_2015_when_notill_yields_more.pdf</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -5993,8 +5802,6 @@
           <t>prinz_2004_microcatchment_swc.pdf</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>paywalled (Elsevier, closed)</t>
@@ -6052,8 +5859,6 @@
           <t>recharge_dam_performance_arid_satellite_2023.pdf</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
           <t>paywalled (Inderscience)</t>
@@ -6103,7 +5908,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/roose_2010_maroc_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/roose_2010_maroc_fr.pdf</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6111,8 +5916,6 @@
           <t>roose_2010_maroc_fr.pdf</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6162,7 +5965,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/roose_2017_restauration_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/roose_2017_restauration_fr.pdf</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6170,8 +5973,6 @@
           <t>roose_2017_restauration_fr.pdf</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6221,7 +6022,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ruzzante_2021.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/ruzzante_2021.pdf</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6229,8 +6030,6 @@
           <t>ruzzante_2021.pdf</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6280,7 +6079,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sawadogo_2011_swc_burkina.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/sawadogo_2011_swc_burkina.pdf</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6288,8 +6087,6 @@
           <t>sawadogo_2011_swc_burkina.pdf</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6339,7 +6136,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/silva_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/silva_2026.pdf</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6347,8 +6144,6 @@
           <t>silva_2026.pdf</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6398,7 +6193,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/steward_2018.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/steward_2018.pdf</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6406,8 +6201,6 @@
           <t>steward_2018.pdf</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6457,7 +6250,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/tadesse_2023_csa_production_risk_review.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/tadesse_2023_csa_production_risk_review.pdf</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6465,8 +6258,6 @@
           <t>tadesse_2023_csa_production_risk_review.pdf</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6516,7 +6307,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/tefera_2024.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/tefera_2024.pdf</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6524,8 +6315,6 @@
           <t>tefera_2024.pdf</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6583,8 +6372,6 @@
           <t>terrace_failure_connectivity_runoff_semiarid_2009.pdf</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>paywalled (Wiley, closed access)</t>
@@ -6634,7 +6421,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/uwizeyimana_2018_water_conservation_rwanda.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/uwizeyimana_2018_water_conservation_rwanda.pdf</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6642,8 +6429,6 @@
           <t>uwizeyimana_2018_water_conservation_rwanda.pdf</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6693,7 +6478,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/wei_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/wei_2016.pdf</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6701,8 +6486,6 @@
           <t>wei_2016.pdf</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6740,7 +6523,6 @@
           <t>Oweis T. et al. / de Winnaar (2014). The potential of in situ rainwater harvesting in arid regions: developing a methodology to identify suitable areas.</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" s="5" t="inlineStr">
         <is>
           <t>https://openalex.org/W2000960672</t>
@@ -6756,8 +6538,6 @@
           <t>wh_insitu_arid_suitability_method_2014.pdf</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>paywalled (closed access); DOI to confirm on retrieval</t>
@@ -6807,7 +6587,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/zhang_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/zhang_2026.pdf</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6815,8 +6595,6 @@
           <t>zhang_2026.pdf</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6866,7 +6644,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/zoure_2025_traditional_practices_burkina.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/zoure_2025_traditional_practices_burkina.pdf</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6874,8 +6652,6 @@
           <t>zoure_2025_traditional_practices_burkina.pdf</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>tool acquisition failed — no candidate URL yielded a PDF (landing page / 403 / no Unpaywall copy); human browser download / OA web-search recovery</t>
@@ -6933,8 +6709,6 @@
           <t>combined_hydro_landscape_2005.pdf</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>paywalled_springer</t>
@@ -6992,8 +6766,6 @@
           <t>dohong_tropical_restoration_techniques_review_2018.pdf</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>paywalled (Springer, closed)</t>
@@ -7051,8 +6823,6 @@
           <t>mcda_two_methods_wetland_2017.pdf</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>paywalled_springer</t>
@@ -7110,8 +6880,6 @@
           <t>oa_instream_wetland_creation_suitability_2025.pdf</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>OA (Unpaywall:None)</t>
@@ -7149,7 +6917,6 @@
           <t>Ramsar Convention (2023). Briefing Note 10: Wetland restoration for climate change resilience.</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" s="5" t="inlineStr">
         <is>
           <t>https://www.ramsar.org/sites/default/files/2023-07/bn10_restoration_climate_change_s.pdf</t>
@@ -7165,8 +6932,6 @@
           <t>ramsar_bn10_restoration_climate_resilience.pdf</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -7209,10 +6974,9 @@
           <t>10.1016/j.jclepro.2022.132768</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/adhikary_2022_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/adhikary_2022_econ.pdf</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7220,8 +6984,6 @@
           <t>adhikary_2022_econ.pdf</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t xml:space="preserve">unpaywall: no OA location (Elsevier) — NOT yet "paywalled": run the required web-search OA recovery (ResearchGate / repository / author copy) before labelling; </t>
@@ -7264,10 +7026,9 @@
           <t>10.1016/j.agee.2020.107175</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bado_2021_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/bado_2021_econ.pdf</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7275,8 +7036,6 @@
           <t>bado_2021_econ.pdf</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t xml:space="preserve">unpaywall: no OA location (Elsevier) — NOT yet "paywalled": run the required web-search OA recovery (ResearchGate / repository / author copy) before labelling; </t>
@@ -7326,7 +7085,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/blackshaw_1994_shade_heat_stress_cattle_review.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/blackshaw_1994_shade_heat_stress_cattle_review.pdf</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7334,8 +7093,6 @@
           <t>blackshaw_1994_shade_heat_stress_cattle_review.pdf</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7385,7 +7142,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/caramori_1996.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/caramori_1996.pdf</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7393,8 +7150,6 @@
           <t>caramori_1996.pdf</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7444,7 +7199,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/de_beenhouwer_2013.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/de_beenhouwer_2013.pdf</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7452,8 +7207,6 @@
           <t>de_beenhouwer_2013.pdf</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7503,7 +7256,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/deniz_2023.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/deniz_2023.pdf</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7511,8 +7264,6 @@
           <t>deniz_2023.pdf</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7562,7 +7313,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/jemaneh_2026.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/jemaneh_2026.pdf</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7570,8 +7321,6 @@
           <t>jemaneh_2026.pdf</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7621,7 +7370,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/julius_2019_rainfall_variability_trees_maize_malawi.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/julius_2019_rainfall_variability_trees_maize_malawi.pdf</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7629,8 +7378,6 @@
           <t>julius_2019_rainfall_variability_trees_maize_malawi.pdf</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7680,7 +7427,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kim_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/kim_2016.pdf</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7688,8 +7435,6 @@
           <t>kim_2016.pdf</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7732,10 +7477,9 @@
           <t>10.1016/j.agsy.2022.103590</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/li_2022_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/li_2022_econ.pdf</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7743,8 +7487,6 @@
           <t>li_2022_econ.pdf</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t xml:space="preserve">unpaywall: no OA location (Elsevier) — NOT yet "paywalled": run the required web-search OA recovery (ResearchGate / repository / author copy) before labelling; </t>
@@ -7794,7 +7536,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/ma_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/ma_2020.pdf</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7802,8 +7544,6 @@
           <t>ma_2020.pdf</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7853,7 +7593,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/mcguigan_2024.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/mcguigan_2024.pdf</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7861,8 +7601,6 @@
           <t>mcguigan_2024.pdf</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -7905,10 +7643,9 @@
           <t>10.1007/s13593-016-0386-6</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/perez_neira_2016_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/perez_neira_2016_econ.pdf</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7916,8 +7653,6 @@
           <t>perez_neira_2016_econ.pdf</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t xml:space="preserve">unpaywall: no OA location (Springer) — NOT yet "paywalled": run the required web-search OA recovery (ResearchGate / repository / author copy) before labelling; </t>
@@ -7967,7 +7702,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sileshi_2008.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/sileshi_2008.pdf</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7975,8 +7710,6 @@
           <t>sileshi_2008.pdf</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8026,7 +7759,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sileshi_2011_legume_trees_yield_stability_agwat.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/sileshi_2011_legume_trees_yield_stability_agwat.pdf</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8034,8 +7767,6 @@
           <t>sileshi_2011_legume_trees_yield_stability_agwat.pdf</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8085,7 +7816,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/sileshi_2012_legume_trees_yield_stability_agronj.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/sileshi_2012_legume_trees_yield_stability_agronj.pdf</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8093,8 +7824,6 @@
           <t>sileshi_2012_legume_trees_yield_stability_agronj.pdf</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8144,7 +7873,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/singh_lal_2018.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/singh_lal_2018.pdf</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8152,8 +7881,6 @@
           <t>singh_lal_2018.pdf</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8203,7 +7930,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/zheng_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/zheng_2020.pdf</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8211,8 +7938,6 @@
           <t>zheng_2020.pdf</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8262,7 +7987,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/akber_2018_sundarbans_storm_protection.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/akber_2018_sundarbans_storm_protection.pdf</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8270,8 +7995,6 @@
           <t>akber_2018_sundarbans_storm_protection.pdf</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8321,7 +8044,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/badola_hussain_2005_bhitarkanika_storm_protection.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/badola_hussain_2005_bhitarkanika_storm_protection.pdf</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8329,8 +8052,6 @@
           <t>badola_hussain_2005_bhitarkanika_storm_protection.pdf</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8380,7 +8101,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/das_2011_mangroves_property_loss_orissa.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/das_2011_mangroves_property_loss_orissa.pdf</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8388,8 +8109,6 @@
           <t>das_2011_mangroves_property_loss_orissa.pdf</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8439,7 +8158,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/woldearegay_2017_landscape_restoration_rwh_ethiopia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/2_ForestRestoration/woldearegay_2017_landscape_restoration_rwh_ethiopia.pdf</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8447,8 +8166,6 @@
           <t>woldearegay_2017_landscape_restoration_rwh_ethiopia.pdf</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8498,7 +8215,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/adimassu_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/adimassu_2016.pdf</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8506,8 +8223,6 @@
           <t>adimassu_2016.pdf</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8545,7 +8260,6 @@
           <t>Arabi, M.; Kedaid, O.E.; Bourougaa, L.; Asla, T.; Roose, É. (2004). Bilan de l'enquête sur la défense et restauration des sols (DRS) en Algérie. Sécheresse, 15(1), 87-95.</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
       <c r="G135" s="5" t="inlineStr">
         <is>
           <t>https://www.researchgate.net/publication/282171205</t>
@@ -8553,7 +8267,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/arabi_2004_drs_algerie_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/arabi_2004_drs_algerie_fr.pdf</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8561,8 +8275,6 @@
           <t>arabi_2004_drs_algerie_fr.pdf</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8612,7 +8324,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/arnaez_2015.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/arnaez_2015.pdf</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8620,8 +8332,6 @@
           <t>arnaez_2015.pdf</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8671,7 +8381,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/barron_okwach_2005_dry_spell_mitigation_kenya.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/barron_okwach_2005_dry_spell_mitigation_kenya.pdf</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8679,8 +8389,6 @@
           <t>barron_okwach_2005_dry_spell_mitigation_kenya.pdf</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8718,11 +8426,9 @@
           <t xml:space="preserve">Botoni, E.; Reij, C. (2009). La transformation silencieuse de l'environnement et des systèmes de production au Sahel : impacts des investissements publics et privés dans la gestion des ressources naturelles. Ouagadougou </t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/botoni_reij_2009_cilss_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/botoni_reij_2009_cilss_fr.pdf</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8730,8 +8436,6 @@
           <t>botoni_reij_2009_cilss_fr.pdf</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8781,7 +8485,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bouma_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/bouma_2016.pdf</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8789,8 +8493,6 @@
           <t>bouma_2016.pdf</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8828,7 +8530,6 @@
           <t>Cárdenas, F.; Taboada, R.; Tafur, J.; Leyva, W.M. (2022). La siembra y cosecha de agua en Apurímac, Ayacucho y Huancavelica: Revisión sistemática de proyectos de desarrollo realizados entre los años 1990 y 2020. Lima: Ce</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" s="5" t="inlineStr">
         <is>
           <t>https://www.researchgate.net/publication/370716126</t>
@@ -8836,7 +8537,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/cardenas_2022_siembra_cosecha_sr_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/cardenas_2022_siembra_cosecha_sr_es.pdf</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8844,8 +8545,6 @@
           <t>cardenas_2022_siembra_cosecha_sr_es.pdf</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8895,7 +8594,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/constenla_2022_land_restoration_drought_ethiopia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/constenla_2022_land_restoration_drought_ethiopia.pdf</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8903,8 +8602,6 @@
           <t>constenla_2022_land_restoration_drought_ethiopia.pdf</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -8954,7 +8651,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/dile_2013.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/dile_2013.pdf</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8962,8 +8659,6 @@
           <t>dile_2013.pdf</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9013,7 +8708,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/fox_rockstrom_2003_si_dry_spell_sahel.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/fox_rockstrom_2003_si_dry_spell_sahel.pdf</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9021,8 +8716,6 @@
           <t>fox_rockstrom_2003_si_dry_spell_sahel.pdf</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9072,7 +8765,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/glendenning_2012.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/glendenning_2012.pdf</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9080,8 +8773,6 @@
           <t>glendenning_2012.pdf</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9131,7 +8822,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kassie_2008_stone_bunds_returns_ethiopia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/kassie_2008_stone_bunds_returns_ethiopia.pdf</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9139,8 +8830,6 @@
           <t>kassie_2008_stone_bunds_returns_ethiopia.pdf</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9190,7 +8879,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kassie_2015_production_risk_malawi.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/kassie_2015_production_risk_malawi.pdf</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9198,8 +8887,6 @@
           <t>kassie_2015_production_risk_malawi.pdf</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9249,7 +8936,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kato_2011.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/kato_2011.pdf</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9257,8 +8944,6 @@
           <t>kato_2011.pdf</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9308,7 +8993,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kidane_2019_ca_production_risk_mozambique.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/kidane_2019_ca_production_risk_mozambique.pdf</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9316,8 +9001,6 @@
           <t>kidane_2019_ca_production_risk_mozambique.pdf</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9367,7 +9050,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/monji_2016_spate_irrigation_drought_tunisia.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/monji_2016_spate_irrigation_drought_tunisia.pdf</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9375,8 +9058,6 @@
           <t>monji_2016_spate_irrigation_drought_tunisia.pdf</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9426,7 +9107,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/rockstrom_2010.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/rockstrom_2010.pdf</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9434,8 +9115,6 @@
           <t>rockstrom_2010.pdf</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9485,7 +9164,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/setimela_2018_el_nino_ca_maize.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/setimela_2018_el_nino_ca_maize.pdf</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9493,8 +9172,6 @@
           <t>setimela_2018_el_nino_ca_maize.pdf</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9544,7 +9221,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/stavi_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/stavi_2020.pdf</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9552,8 +9229,6 @@
           <t>stavi_2020.pdf</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9603,7 +9278,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/thierfelder_2026_ca_dt_bundling_zimbabwe.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/thierfelder_2026_ca_dt_bundling_zimbabwe.pdf</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9611,8 +9286,6 @@
           <t>thierfelder_2026_ca_dt_bundling_zimbabwe.pdf</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9662,7 +9335,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/thierfelder_wall_2010_ca_zambia_zimbabwe.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/thierfelder_wall_2010_ca_zambia_zimbabwe.pdf</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9670,8 +9343,6 @@
           <t>thierfelder_wall_2010_ca_zambia_zimbabwe.pdf</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9721,7 +9392,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/waqas_2025_rwh_drought_mitigation.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/waqas_2025_rwh_drought_mitigation.pdf</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9729,8 +9400,6 @@
           <t>waqas_2025_rwh_drought_mitigation.pdf</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>OA (websearch:researchgate/unverified) — HUMAN CHECK</t>
@@ -9780,7 +9449,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/chausson_2020.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/chausson_2020.pdf</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9788,8 +9457,6 @@
           <t>chausson_2020.pdf</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -9839,7 +9506,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/cisneros_2024_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/cisneros_2024_es.pdf</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -9847,8 +9514,6 @@
           <t>cisneros_2024_es.pdf</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -9898,7 +9563,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/coulibaly_2016_icraf_wp223.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/coulibaly_2016_icraf_wp223.pdf</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9906,8 +9571,6 @@
           <t>coulibaly_2016_icraf_wp223.pdf</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -9957,7 +9620,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/damianidis_2021.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/damianidis_2021.pdf</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9965,8 +9628,6 @@
           <t>damianidis_2021.pdf</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -10016,7 +9677,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/lasco_2014.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/lasco_2014.pdf</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10024,8 +9685,6 @@
           <t>lasco_2014.pdf</t>
         </is>
       </c>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -10063,7 +9722,6 @@
           <t>Montagnini, F.; Somarriba, E.; Murgueitio, E.; Fassola, H.; Eibl, B. (eds.) (2015). Sistemas agroforestales. Funciones productivas, socioeconómicas y ambientales. CATIE (Turrialba) / CIPAV (Cali). [series number to confi</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
       <c r="G161" s="5" t="inlineStr">
         <is>
           <t>https://repositorio.catie.ac.cr/bitstream/handle/11554/7124/Sistemas_Agroforestales.pdf?sequence=1</t>
@@ -10071,7 +9729,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/montagnini_2015_catie_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/montagnini_2015_catie_es.pdf</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10079,8 +9737,6 @@
           <t>montagnini_2015_catie_es.pdf</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -10130,7 +9786,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/quenol_2006_fr.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/quenol_2006_fr.pdf</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10138,8 +9794,6 @@
           <t>quenol_2006_fr.pdf</t>
         </is>
       </c>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -10189,7 +9843,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/shi_2018.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/shi_2018.pdf</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10197,8 +9851,6 @@
           <t>shi_2018.pdf</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block — human browser download from publisher/repository URL</t>
@@ -10236,11 +9888,9 @@
           <t>Said, M. T.; Ameen, F. A. (2016). Effect of Sowing Methods and Microelements Foliar Application on Bread Wheat Productivity and their Economical Feasibility. Egyptian Journal of Agronomy.</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_eo0122_said_2016.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_eo0122_said_2016.pdf</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10248,8 +9898,6 @@
           <t>era_eo0122_said_2016.pdf</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
         <is>
           <t>tool acquisition failed — no URL/DOI route; human browser download / OA web-search recovery</t>
@@ -10287,11 +9935,9 @@
           <t>Abubaker, B. M. A.; Yu, S. E.; Shao, G. C.; Alhadi, M. (2014). IMPACT OF DIFFERENT WATER HARVESTING TECHNIQUES ON SOIL MOISTURE CONTENT AND YIELD COMPONENTS OF SORGHUM. Pakistan Journal of Agricultural Sciences.</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/era_nj0007_abubaker_2014.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/era_nj0007_abubaker_2014.pdf</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10299,8 +9945,6 @@
           <t>era_nj0007_abubaker_2014.pdf</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr">
         <is>
           <t>tool acquisition failed — no URL/DOI route; human browser download / OA web-search recovery</t>
@@ -10358,8 +10002,6 @@
           <t>wet_catchment_es_suitability_ecoind_2017.pdf</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10417,8 +10059,6 @@
           <t>wet_feasible_locations_lidar_suitability_2018.pdf</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10476,8 +10116,6 @@
           <t>wet_global_potential_climate_ensemble_2025.pdf</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10535,8 +10173,6 @@
           <t>wet_mcda_suitability_index_ontario_2020.pdf</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10594,8 +10230,6 @@
           <t>wet_potential_distribution_china_ml_2023.pdf</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
       <c r="L170" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10653,8 +10287,6 @@
           <t>wet_potential_restoration_indicator_conus_2017.pdf</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10712,8 +10344,6 @@
           <t>wet_potential_wetlands_rf_bigdata_2023.pdf</t>
         </is>
       </c>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10771,8 +10401,6 @@
           <t>wet_rehabilitation_areas_multisource_china_2020.pdf</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr"/>
-      <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr">
         <is>
           <t>webfetch_403_bot_block</t>
@@ -10822,7 +10450,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/aiyelaagbe_2001_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/aiyelaagbe_2001_econ.pdf</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10830,9 +10458,6 @@
           <t>aiyelaagbe_2001_econ.pdf</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
       <c r="M174" t="inlineStr">
         <is>
           <t>aiyelaagbe_2001_econ</t>
@@ -10877,7 +10502,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/bucagu_2013_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/bucagu_2013_econ.pdf</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10885,9 +10510,6 @@
           <t>bucagu_2013_econ.pdf</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr">
         <is>
           <t>bucagu_2013_econ</t>
@@ -10920,7 +10542,6 @@
           <t>Current, D.; Lutz, E.; Scherr, S.J. ([year to confirm]). Adopción agrícola y beneficios económicos de la agroforestería: experiencias en América Central y el Caribe. [Spanish edition; publisher/year to confirm from CATIE</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
       <c r="G176" s="5" t="inlineStr">
         <is>
           <t>http://repositorio.bibliotecaorton.catie.ac.cr/handle/11554/129</t>
@@ -10928,7 +10549,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/current_1995_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/current_1995_es.pdf</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -10936,8 +10557,6 @@
           <t>current_1995_es.pdf</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
         <is>
           <t>publisher URL dead/unreachable — locate copy (repository / author / library)</t>
@@ -10987,7 +10606,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/fadl_2013_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/fadl_2013_econ.pdf</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10995,9 +10614,6 @@
           <t>fadl_2013_econ.pdf</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr">
         <is>
           <t>fadl_2013_econ</t>
@@ -11030,7 +10646,6 @@
           <t>Haglund et al. (2011). Dry land tree management for improved household livelihoods: Farmer managed natural regeneration in Niger. Journal of Environmental Management.</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" s="5" t="inlineStr">
         <is>
           <t>https://oar.icrisat.org/1659/</t>
@@ -11046,8 +10661,6 @@
           <t>haglund_2011.pdf</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
         <is>
           <t>OA (websearch:agency-repo/med)</t>
@@ -11097,7 +10710,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/kormawa_1999_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/kormawa_1999_econ.pdf</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11105,9 +10718,6 @@
           <t>kormawa_1999_econ.pdf</t>
         </is>
       </c>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
       <c r="M179" t="inlineStr">
         <is>
           <t>kormawa_1999_econ</t>
@@ -11152,7 +10762,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/maliki_2012_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/maliki_2012_econ.pdf</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11160,9 +10770,6 @@
           <t>maliki_2012_econ.pdf</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr">
         <is>
           <t>maliki_2012_econ</t>
@@ -11207,7 +10814,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/midega_2014_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/midega_2014_econ.pdf</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11215,9 +10822,6 @@
           <t>midega_2014_econ.pdf</t>
         </is>
       </c>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
       <c r="M181" t="inlineStr">
         <is>
           <t>midega_2014_econ</t>
@@ -11262,7 +10866,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/navas_2010_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/navas_2010_es.pdf</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -11270,8 +10874,6 @@
           <t>navas_2010_es.pdf</t>
         </is>
       </c>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
       <c r="L182" t="inlineStr">
         <is>
           <t>publisher URL dead/unreachable — locate copy (repository / author / library)</t>
@@ -11321,7 +10923,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/onduru_2008_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/onduru_2008_econ.pdf</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -11329,9 +10931,6 @@
           <t>onduru_2008_econ.pdf</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr">
         <is>
           <t>onduru_2008_econ</t>
@@ -11364,7 +10963,6 @@
           <t>Reyes, T.;Quiroz, R.;Msikula, S. (2005). Socio-economic comparison between traditional and improved cultivation methods in agroforestry systems, East Usambara Mountains, Tanzania. Environmental Management.</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" s="5" t="inlineStr">
         <is>
           <t>NA</t>
@@ -11372,7 +10970,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/reyes_2005_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/reyes_2005_econ.pdf</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -11380,9 +10978,6 @@
           <t>reyes_2005_econ.pdf</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr">
         <is>
           <t>reyes_2005_econ</t>
@@ -11427,7 +11022,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/saucedo_2023_es.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/saucedo_2023_es.pdf</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -11435,8 +11030,6 @@
           <t>saucedo_2023_es.pdf</t>
         </is>
       </c>
-      <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr">
         <is>
           <t>publisher URL dead/unreachable — locate copy (repository / author / library)</t>
@@ -11474,7 +11067,6 @@
           <t>(2023). Shade versus intensification: trade-off or synergy for profitability in coffee agroforestry systems? (OpenAlex W4389586869).</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
       <c r="G186" s="5" t="inlineStr">
         <is>
           <t>https://gala.gre.ac.uk/id/eprint/45113/13/45113_LALANI_%20Shade_versus_intensification_Trade_off_or_synergy.pdf</t>
@@ -11490,8 +11082,6 @@
           <t>shade_vs_intensification_2023_profitability.pdf</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
       <c r="L186" t="inlineStr">
         <is>
           <t>OA (websearch:university-repo/high)</t>
@@ -11529,7 +11119,6 @@
           <t>Herbage production during drought in silvopastoral systems on a rocky rangeland in arid zone of India. Annals of Arid Zone 47(1) (2008).</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr"/>
       <c r="G187" s="5" t="inlineStr">
         <is>
           <t>https://ijoear.com/assets/resources/naas-journal-rating-2025.pdf</t>
@@ -11545,8 +11134,6 @@
           <t>silvopastoral_drought_herbage_arid_india_2008.pdf</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr">
         <is>
           <t>title verification failed on the cached 95-page file (journal volume, not the article) — re-acquire the article by title (2026-10-06)</t>
@@ -11596,7 +11183,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/snapp_2010_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/snapp_2010_econ.pdf</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -11604,9 +11191,6 @@
           <t>snapp_2010_econ.pdf</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr">
         <is>
           <t>snapp_2010_econ</t>
@@ -11651,7 +11235,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/tonye_1995_econ.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/1_Agroforestry/tonye_1995_econ.pdf</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -11659,9 +11243,6 @@
           <t>tonye_1995_econ.pdf</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr">
         <is>
           <t>tonye_1995_econ</t>
@@ -11694,7 +11275,6 @@
           <t>Meta-analysis of carbon stocks and biodiversity outcomes across Brazilian restored biomes, Science of the Total Environment (2023), S0048969723061855</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr"/>
       <c r="G190" s="5" t="inlineStr">
         <is>
           <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4510899</t>
@@ -11710,8 +11290,6 @@
           <t>brazil_biomes_carbon_biodiv_meta_2023.pdf</t>
         </is>
       </c>
-      <c r="J190" t="inlineStr"/>
-      <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr">
         <is>
           <t>OA (websearch:ssrn/med)</t>
@@ -11769,8 +11347,6 @@
           <t>nat_rev_biodiv_nr_drivers.pdf</t>
         </is>
       </c>
-      <c r="J191" t="inlineStr"/>
-      <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
         <is>
           <t>OA (websearch:wur/med)</t>
@@ -11828,8 +11404,6 @@
           <t>spruce_drought_succession.pdf</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr">
         <is>
           <t>OA (websearch:academia/med)</t>
@@ -11867,7 +11441,6 @@
           <t>Oweis, T.; Prinz, D.; Hachum, A. (2001). Water harvesting: indigenous knowledge for the future of the drier environments. ICARDA, Aleppo.</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
       <c r="G193" s="5" t="inlineStr">
         <is>
           <t>https://mel.cgiar.org/reporting/downloadmelspace/hash/8822931d10e9b1436357e37cc0ad95ef/v/699ed9daff637546058c1c3544115468</t>
@@ -11875,7 +11448,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/&lt;NbS folder&gt;/icarda_oweis_wh_indigenous_2001.pdf</t>
+          <t>D591_Rural-Scan_NBS/2_Technical_&amp;_Data/library/3_Water_Harvesting/icarda_oweis_wh_indigenous_2001.pdf</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -11883,8 +11456,6 @@
           <t>icarda_oweis_wh_indigenous_2001.pdf</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
       <c r="L193" t="inlineStr">
         <is>
           <t>needs_ocr (scanned PDF, no text layer)</t>

</xml_diff>